<commit_message>
Cimentación: hormigón aparte a 95 €/m³ y acero aparte
Suministro de HA-25 a 95 €/m³ sobre los 37 m³ (3.515 €): la cimentación
va por 10.400,30 € sin IVA con la mano de obra del equipo. El suministro
de acero queda como partida aparte, con el precio pendiente.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UsshWDyzh9XkyW9ZdDTfjF
</commit_message>
<xml_diff>
--- a/costes/Nevola_cimentacion_presupuesto_equipo.xlsx
+++ b/costes/Nevola_cimentacion_presupuesto_equipo.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="95">
   <si>
     <t xml:space="preserve">Névola · Cimentación del piloto · Presupuesto del equipo</t>
   </si>
@@ -102,7 +102,7 @@
     <t xml:space="preserve">Lo que no aparece en el manuscrito (a confirmar con el equipo)</t>
   </si>
   <si>
-    <t xml:space="preserve">Los precios del manuscrito parecen de mano de obra: encofrado por metro, vertido (no suministro) a 16,50 €/m³ y armado por kg. Si es así, faltan los materiales y el movimiento de tierras. Precios en blanco: rellenar cuando el equipo los confirme.</t>
+    <t xml:space="preserve">Los precios del manuscrito son de mano de obra: encofrado por metro, vertido (no suministro) a 16,50 €/m³ y armado por kg. El hormigón se suministra aparte a 95 €/m³ y el acero también va aparte. Precios en blanco: rellenar cuando estén confirmados.</t>
   </si>
   <si>
     <t xml:space="preserve">De dónde sale la cantidad</t>
@@ -111,13 +111,13 @@
     <t xml:space="preserve">Suministro de hormigón HA-25</t>
   </si>
   <si>
-    <t xml:space="preserve">Los 37 m³ vertidos</t>
+    <t xml:space="preserve">Los 37 m³ vertidos. Precio de Iván (20/10/2026)</t>
   </si>
   <si>
     <t xml:space="preserve">Suministro de acero B500S</t>
   </si>
   <si>
-    <t xml:space="preserve">Si los 0,67 €/kg son solo elaboración y armado</t>
+    <t xml:space="preserve">Va aparte de los 0,67 €/kg de elaboración y armado. Precio pendiente</t>
   </si>
   <si>
     <t xml:space="preserve">Hormigón de limpieza bajo zapatas</t>
@@ -285,10 +285,7 @@
     <t xml:space="preserve">Antes de darlo por bueno.</t>
   </si>
   <si>
-    <t xml:space="preserve">¿Los precios son solo de mano de obra? ¿Incluyen el suministro de hormigón HA-25 y de acero, o van aparte?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Los 0,67 €/kg del hierro: ¿son elaboración y armado, o también el suministro del acero?</t>
+    <t xml:space="preserve">Hormigón y acero van aparte (hormigón a 95 €/m³). ¿A qué precio está el acero B500S suministrado en obra?</t>
   </si>
   <si>
     <t xml:space="preserve">¿Quién hace y paga la excavación de zanjas, la retirada de tierras, el hormigón de limpieza y la grava de la cámara sanitaria?</t>
@@ -1061,7 +1058,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4"/>
       <c r="B17" s="4" t="s">
         <v>28</v>
@@ -1076,13 +1073,15 @@
         <f aca="false">E7+E8</f>
         <v>37</v>
       </c>
-      <c r="F17" s="6"/>
-      <c r="G17" s="7" t="str">
+      <c r="F17" s="6" t="n">
+        <v>95</v>
+      </c>
+      <c r="G17" s="7" t="n">
         <f aca="false">IF(F17="","",E17*F17)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>3515</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4"/>
       <c r="B18" s="4" t="s">
         <v>30</v>
@@ -1202,7 +1201,7 @@
       </c>
       <c r="G24" s="15" t="n">
         <f aca="false">SUM(G17:G23)</f>
-        <v>0</v>
+        <v>3515</v>
       </c>
     </row>
     <row r="25" s="8" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1211,7 +1210,7 @@
       </c>
       <c r="G25" s="10" t="n">
         <f aca="false">G11+G24</f>
-        <v>6885.3</v>
+        <v>10400.3</v>
       </c>
     </row>
   </sheetData>
@@ -1596,7 +1595,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -1621,7 +1620,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="n">
         <v>2</v>
       </c>
@@ -1629,7 +1628,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="n">
         <v>3</v>
       </c>
@@ -1637,7 +1636,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="n">
         <v>4</v>
       </c>
@@ -1645,7 +1644,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="n">
         <v>5</v>
       </c>
@@ -1653,7 +1652,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="n">
         <v>6</v>
       </c>
@@ -1661,7 +1660,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="n">
         <v>7</v>
       </c>
@@ -1675,14 +1674,6 @@
       </c>
       <c r="B11" s="4" t="s">
         <v>94</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cimentación: acero aparte a 0,95 €/kg
3.000 kg de B500S a 0,95 €/kg (2.850 €). Con mano de obra, hormigón y
acero, la cimentación va por 13.250,30 € sin IVA.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UsshWDyzh9XkyW9ZdDTfjF
</commit_message>
<xml_diff>
--- a/costes/Nevola_cimentacion_presupuesto_equipo.xlsx
+++ b/costes/Nevola_cimentacion_presupuesto_equipo.xlsx
@@ -102,7 +102,7 @@
     <t xml:space="preserve">Lo que no aparece en el manuscrito (a confirmar con el equipo)</t>
   </si>
   <si>
-    <t xml:space="preserve">Los precios del manuscrito son de mano de obra: encofrado por metro, vertido (no suministro) a 16,50 €/m³ y armado por kg. El hormigón se suministra aparte a 95 €/m³ y el acero también va aparte. Precios en blanco: rellenar cuando estén confirmados.</t>
+    <t xml:space="preserve">Los precios del manuscrito son de mano de obra: encofrado por metro, vertido (no suministro) a 16,50 €/m³ y armado por kg. El hormigón (95 €/m³) y el acero (0,95 €/kg) se suministran aparte. Precios en blanco: rellenar cuando estén confirmados.</t>
   </si>
   <si>
     <t xml:space="preserve">De dónde sale la cantidad</t>
@@ -117,7 +117,7 @@
     <t xml:space="preserve">Suministro de acero B500S</t>
   </si>
   <si>
-    <t xml:space="preserve">Va aparte de los 0,67 €/kg de elaboración y armado. Precio pendiente</t>
+    <t xml:space="preserve">Los 3.000 kg, aparte de los 0,67 €/kg de elaboración y armado. Precio de Iván (20/10/2026)</t>
   </si>
   <si>
     <t xml:space="preserve">Hormigón de limpieza bajo zapatas</t>
@@ -285,7 +285,7 @@
     <t xml:space="preserve">Antes de darlo por bueno.</t>
   </si>
   <si>
-    <t xml:space="preserve">Hormigón y acero van aparte (hormigón a 95 €/m³). ¿A qué precio está el acero B500S suministrado en obra?</t>
+    <t xml:space="preserve">Hormigón (95 €/m³) y acero (0,95 €/kg) van aparte. ¿Confirmáis que vuestro precio no incluye ningún material salvo las placas?</t>
   </si>
   <si>
     <t xml:space="preserve">¿Quién hace y paga la excavación de zanjas, la retirada de tierras, el hormigón de limpieza y la grava de la cámara sanitaria?</t>
@@ -1096,10 +1096,12 @@
         <f aca="false">E9</f>
         <v>3000</v>
       </c>
-      <c r="F18" s="6"/>
-      <c r="G18" s="7" t="str">
+      <c r="F18" s="6" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="G18" s="7" t="n">
         <f aca="false">IF(F18="","",E18*F18)</f>
-        <v/>
+        <v>2850</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1201,7 +1203,7 @@
       </c>
       <c r="G24" s="15" t="n">
         <f aca="false">SUM(G17:G23)</f>
-        <v>3515</v>
+        <v>6365</v>
       </c>
     </row>
     <row r="25" s="8" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1210,7 +1212,7 @@
       </c>
       <c r="G25" s="10" t="n">
         <f aca="false">G11+G24</f>
-        <v>10400.3</v>
+        <v>13250.3</v>
       </c>
     </row>
   </sheetData>
@@ -1612,7 +1614,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="n">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
Cimentación: hormigón de limpieza a 9 €/m²
45,75 m² bajo zapatas a 9 €/m² (411,75 €). La cimentación va por
13.662,05 € sin IVA.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UsshWDyzh9XkyW9ZdDTfjF
</commit_message>
<xml_diff>
--- a/costes/Nevola_cimentacion_presupuesto_equipo.xlsx
+++ b/costes/Nevola_cimentacion_presupuesto_equipo.xlsx
@@ -123,7 +123,7 @@
     <t xml:space="preserve">Hormigón de limpieza bajo zapatas</t>
   </si>
   <si>
-    <t xml:space="preserve">Superficie de zapatas del croquis: 10,00 × (0,75 + 0,90 + 0,90 + 0,75) + 2 × 8,50 × 0,75</t>
+    <t xml:space="preserve">Superficie de zapatas del croquis: 10,00 × (0,75 + 0,90 + 0,90 + 0,75) + 2 × 8,50 × 0,75. Precio de Iván (20/10/2026)</t>
   </si>
   <si>
     <t xml:space="preserve">m²</t>
@@ -1104,7 +1104,7 @@
         <v>2850</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4"/>
       <c r="B19" s="4" t="s">
         <v>32</v>
@@ -1119,10 +1119,12 @@
         <f aca="false">10*(0.75+0.9+0.9+0.75)+2*8.5*0.75</f>
         <v>45.75</v>
       </c>
-      <c r="F19" s="6"/>
-      <c r="G19" s="7" t="str">
+      <c r="F19" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G19" s="7" t="n">
         <f aca="false">IF(F19="","",E19*F19)</f>
-        <v/>
+        <v>411.75</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1203,7 +1205,7 @@
       </c>
       <c r="G24" s="15" t="n">
         <f aca="false">SUM(G17:G23)</f>
-        <v>6365</v>
+        <v>6776.75</v>
       </c>
     </row>
     <row r="25" s="8" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1212,7 +1214,7 @@
       </c>
       <c r="G25" s="10" t="n">
         <f aca="false">G11+G24</f>
-        <v>13250.3</v>
+        <v>13662.05</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cimentación: excavación a 18 €/m³
59,48 m³ (superficie de zapatas × 1,30 m de fondo, por confirmar) a
18 €/m³: 1.070,55 €. La cimentación va por 14.732,60 € sin IVA.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UsshWDyzh9XkyW9ZdDTfjF
</commit_message>
<xml_diff>
--- a/costes/Nevola_cimentacion_presupuesto_equipo.xlsx
+++ b/costes/Nevola_cimentacion_presupuesto_equipo.xlsx
@@ -132,7 +132,7 @@
     <t xml:space="preserve">Excavación de zanjas y retirada de tierras</t>
   </si>
   <si>
-    <t xml:space="preserve">Pendiente de medir</t>
+    <t xml:space="preserve">Superficie de zapatas (45,75 m²) × 1,30 m de fondo, como en la estimación A (coronación a −0,05, muro, zapata y limpieza). Sin descontar cruces. Precio de Iván (20/10/2026)</t>
   </si>
   <si>
     <t xml:space="preserve">Grava o lámina en la cámara sanitaria</t>
@@ -1127,7 +1127,7 @@
         <v>411.75</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4"/>
       <c r="B20" s="4" t="s">
         <v>35</v>
@@ -1138,11 +1138,16 @@
       <c r="D20" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="E20" s="5"/>
-      <c r="F20" s="6"/>
-      <c r="G20" s="7" t="str">
+      <c r="E20" s="5" t="n">
+        <f aca="false">(10*(0.75+0.9+0.9+0.75)+2*8.5*0.75)*1.3</f>
+        <v>59.475</v>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="G20" s="7" t="n">
         <f aca="false">IF(F20="","",E20*F20)</f>
-        <v/>
+        <v>1070.55</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1205,7 +1210,7 @@
       </c>
       <c r="G24" s="15" t="n">
         <f aca="false">SUM(G17:G23)</f>
-        <v>6776.75</v>
+        <v>7847.3</v>
       </c>
     </row>
     <row r="25" s="8" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1214,7 +1219,7 @@
       </c>
       <c r="G25" s="10" t="n">
         <f aca="false">G11+G24</f>
-        <v>13662.05</v>
+        <v>14732.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cimentación: grava de cámara sanitaria a 12 €/m²
74,58 m² (huella de planta baja, 7,85 × 9,50) a 12 €/m²: 894,90 €. La
cimentación va por 15.627,50 € sin IVA.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UsshWDyzh9XkyW9ZdDTfjF
</commit_message>
<xml_diff>
--- a/costes/Nevola_cimentacion_presupuesto_equipo.xlsx
+++ b/costes/Nevola_cimentacion_presupuesto_equipo.xlsx
@@ -135,10 +135,10 @@
     <t xml:space="preserve">Superficie de zapatas (45,75 m²) × 1,30 m de fondo, como en la estimación A (coronación a −0,05, muro, zapata y limpieza). Sin descontar cruces. Precio de Iván (20/10/2026)</t>
   </si>
   <si>
-    <t xml:space="preserve">Grava o lámina en la cámara sanitaria</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pendiente de definir</t>
+    <t xml:space="preserve">Grava en la cámara sanitaria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Huella de planta baja: 7,85 × 9,50 m, sin descontar muros, como en la estimación A. Precio de Iván (20/10/2026)</t>
   </si>
   <si>
     <t xml:space="preserve">Bombeo de hormigón</t>
@@ -1150,7 +1150,7 @@
         <v>1070.55</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4"/>
       <c r="B21" s="4" t="s">
         <v>37</v>
@@ -1161,11 +1161,16 @@
       <c r="D21" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="E21" s="5"/>
-      <c r="F21" s="6"/>
-      <c r="G21" s="7" t="str">
+      <c r="E21" s="5" t="n">
+        <f aca="false">7.85*9.5</f>
+        <v>74.575</v>
+      </c>
+      <c r="F21" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="G21" s="7" t="n">
         <f aca="false">IF(F21="","",E21*F21)</f>
-        <v/>
+        <v>894.9</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1210,7 +1215,7 @@
       </c>
       <c r="G24" s="15" t="n">
         <f aca="false">SUM(G17:G23)</f>
-        <v>7847.3</v>
+        <v>8742.2</v>
       </c>
     </row>
     <row r="25" s="8" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1219,7 +1224,7 @@
       </c>
       <c r="G25" s="10" t="n">
         <f aca="false">G11+G24</f>
-        <v>14732.6</v>
+        <v>15627.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cimentación: hormigón a 115 €/m³ y solera de limpieza en mano de obra
Hormigón HA-25 a 115 €/m³; el hormigón de limpieza pasa a 11,50 €/m²
(10 cm al precio del hormigón, enlazado en el Excel). La mano de obra
suma la solera de limpieza a 11 €/m² (503,25 €). Total por vivienda:
16.985,13 € sin IVA, también en /cimentacion/.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UsshWDyzh9XkyW9ZdDTfjF
</commit_message>
<xml_diff>
--- a/costes/Nevola_cimentacion_presupuesto_equipo.xlsx
+++ b/costes/Nevola_cimentacion_presupuesto_equipo.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="97">
   <si>
     <t xml:space="preserve">Névola · Cimentación del piloto · Presupuesto del equipo</t>
   </si>
@@ -93,10 +93,19 @@
     <t xml:space="preserve">ud</t>
   </si>
   <si>
+    <t xml:space="preserve">Solera de limpieza (mano de obra)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Superficie de zapatas del croquis. Añadida por Iván (20/10/2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">m²</t>
+  </si>
+  <si>
     <t xml:space="preserve">Total del presupuesto del equipo</t>
   </si>
   <si>
-    <t xml:space="preserve">En el manuscrito: 6.885,00 €. La diferencia son los redondeos (1.144,80 → 1.145 y 610,50 → 610).</t>
+    <t xml:space="preserve">En el manuscrito: 6.885,00 €, sin la solera de limpieza, que se añadió después. Los céntimos son redondeos del papel (1.144,80 → 1.145 y 610,50 → 610).</t>
   </si>
   <si>
     <t xml:space="preserve">Lo que no aparece en el manuscrito (a confirmar con el equipo)</t>
@@ -123,10 +132,7 @@
     <t xml:space="preserve">Hormigón de limpieza bajo zapatas</t>
   </si>
   <si>
-    <t xml:space="preserve">Superficie de zapatas del croquis: 10,00 × (0,75 + 0,90 + 0,90 + 0,75) + 2 × 8,50 × 0,75. Precio de Iván (20/10/2026)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">m²</t>
+    <t xml:space="preserve">Superficie de zapatas del croquis: 10,00 × (0,75 + 0,90 + 0,90 + 0,75) + 2 × 8,50 × 0,75. Precio: 10 cm de espesor al precio del hormigón</t>
   </si>
   <si>
     <t xml:space="preserve">Excavación de zanjas y retirada de tierras</t>
@@ -817,7 +823,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -1007,127 +1013,129 @@
         <v>384</v>
       </c>
     </row>
-    <row r="11" s="8" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="9" t="s">
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="G11" s="10" t="n">
-        <f aca="false">SUM(G5:G10)</f>
-        <v>6885.3</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="11" t="s">
+      <c r="C11" s="4" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="12" t="s">
+      <c r="D11" s="4" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="15" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="13" t="s">
+      <c r="E11" s="5" t="n">
+        <f aca="false">10*(0.75+0.9+0.9+0.75)+2*8.5*0.75</f>
+        <v>45.75</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="G11" s="7" t="n">
+        <f aca="false">E11*F11</f>
+        <v>503.25</v>
+      </c>
+    </row>
+    <row r="12" s="8" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="B15" s="13"/>
-      <c r="C15" s="13"/>
-      <c r="D15" s="13"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13"/>
-      <c r="G15" s="13"/>
-    </row>
-    <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3"/>
-      <c r="B16" s="3" t="s">
+      <c r="G12" s="10" t="n">
+        <f aca="false">SUM(G5:G11)</f>
+        <v>7388.55</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="12" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" s="13"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="13"/>
+      <c r="F16" s="13"/>
+      <c r="G16" s="13"/>
+    </row>
+    <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3"/>
+      <c r="B17" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C16" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="D16" s="3" t="s">
+      <c r="C17" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D17" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="E17" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="F17" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="G16" s="3" t="s">
+      <c r="G17" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4"/>
-      <c r="B17" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D17" s="4" t="s">
+    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4"/>
+      <c r="B18" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D18" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="E17" s="5" t="n">
+      <c r="E18" s="5" t="n">
         <f aca="false">E7+E8</f>
         <v>37</v>
       </c>
-      <c r="F17" s="6" t="n">
-        <v>95</v>
-      </c>
-      <c r="G17" s="7" t="n">
-        <f aca="false">IF(F17="","",E17*F17)</f>
-        <v>3515</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4"/>
-      <c r="B18" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="D18" s="4" t="s">
+      <c r="F18" s="6" t="n">
+        <v>115</v>
+      </c>
+      <c r="G18" s="7" t="n">
+        <f aca="false">IF(F18="","",E18*F18)</f>
+        <v>4255</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4"/>
+      <c r="B19" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D19" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E18" s="5" t="n">
+      <c r="E19" s="5" t="n">
         <f aca="false">E9</f>
         <v>3000</v>
       </c>
-      <c r="F18" s="6" t="n">
+      <c r="F19" s="6" t="n">
         <v>0.95</v>
-      </c>
-      <c r="G18" s="7" t="n">
-        <f aca="false">IF(F18="","",E18*F18)</f>
-        <v>2850</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4"/>
-      <c r="B19" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="E19" s="5" t="n">
-        <f aca="false">10*(0.75+0.9+0.9+0.75)+2*8.5*0.75</f>
-        <v>45.75</v>
-      </c>
-      <c r="F19" s="6" t="n">
-        <v>9</v>
       </c>
       <c r="G19" s="7" t="n">
         <f aca="false">IF(F19="","",E19*F19)</f>
-        <v>411.75</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>2850</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4"/>
       <c r="B20" s="4" t="s">
         <v>35</v>
@@ -1136,21 +1144,22 @@
         <v>36</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="E20" s="5" t="n">
-        <f aca="false">(10*(0.75+0.9+0.9+0.75)+2*8.5*0.75)*1.3</f>
-        <v>59.475</v>
+        <f aca="false">10*(0.75+0.9+0.9+0.75)+2*8.5*0.75</f>
+        <v>45.75</v>
       </c>
       <c r="F20" s="6" t="n">
-        <v>18</v>
+        <f aca="false">0.1*F18</f>
+        <v>11.5</v>
       </c>
       <c r="G20" s="7" t="n">
         <f aca="false">IF(F20="","",E20*F20)</f>
-        <v>1070.55</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>526.125</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4"/>
       <c r="B21" s="4" t="s">
         <v>37</v>
@@ -1159,21 +1168,21 @@
         <v>38</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="E21" s="5" t="n">
-        <f aca="false">7.85*9.5</f>
-        <v>74.575</v>
+        <f aca="false">(10*(0.75+0.9+0.9+0.75)+2*8.5*0.75)*1.3</f>
+        <v>59.475</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="G21" s="7" t="n">
         <f aca="false">IF(F21="","",E21*F21)</f>
-        <v>894.9</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1070.55</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4"/>
       <c r="B22" s="4" t="s">
         <v>39</v>
@@ -1182,13 +1191,18 @@
         <v>40</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="E22" s="5"/>
-      <c r="F22" s="6"/>
-      <c r="G22" s="7" t="str">
+        <v>25</v>
+      </c>
+      <c r="E22" s="5" t="n">
+        <f aca="false">7.85*9.5</f>
+        <v>74.575</v>
+      </c>
+      <c r="F22" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="G22" s="7" t="n">
         <f aca="false">IF(F22="","",E22*F22)</f>
-        <v/>
+        <v>894.9</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1209,27 +1223,45 @@
         <v/>
       </c>
     </row>
-    <row r="24" s="14" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="14" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4"/>
+      <c r="B24" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="G24" s="15" t="n">
-        <f aca="false">SUM(G17:G23)</f>
-        <v>8742.2</v>
-      </c>
-    </row>
-    <row r="25" s="8" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="9" t="s">
+      <c r="C24" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="G25" s="10" t="n">
-        <f aca="false">G11+G24</f>
-        <v>15627.5</v>
+      <c r="D24" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E24" s="5"/>
+      <c r="F24" s="6"/>
+      <c r="G24" s="7" t="str">
+        <f aca="false">IF(F24="","",E24*F24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" s="14" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="G25" s="15" t="n">
+        <f aca="false">SUM(G18:G24)</f>
+        <v>9596.575</v>
+      </c>
+    </row>
+    <row r="26" s="8" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="G26" s="10" t="n">
+        <f aca="false">G12+G25</f>
+        <v>16985.125</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A15:G15"/>
+    <mergeCell ref="A16:G16"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1256,34 +1288,34 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B5" s="16" t="n">
         <f aca="false">'Presupuesto equipo'!E7</f>
@@ -1297,12 +1329,12 @@
         <v>2.42</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B6" s="16" t="n">
         <f aca="false">'Presupuesto equipo'!E8</f>
@@ -1316,12 +1348,12 @@
         <v>5.52</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B7" s="16" t="n">
         <f aca="false">B5+B6</f>
@@ -1339,7 +1371,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B8" s="17" t="n">
         <f aca="false">'Presupuesto equipo'!E9</f>
@@ -1353,12 +1385,12 @@
         <v>1333</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B9" s="16" t="n">
         <f aca="false">B8/B7</f>
@@ -1373,12 +1405,12 @@
         <v>23.7170067521066</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B10" s="17" t="n">
         <f aca="false">'Presupuesto equipo'!E10</f>
@@ -1392,12 +1424,12 @@
         <v>-6</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B11" s="16" t="n">
         <v>0.7</v>
@@ -1413,7 +1445,7 @@
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B12" s="16" t="n">
         <v>7.95</v>
@@ -1426,20 +1458,20 @@
         <v>1.05</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
@@ -1447,10 +1479,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C16" s="4"/>
       <c r="D16" s="4"/>
@@ -1458,10 +1490,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C17" s="4"/>
       <c r="D17" s="4"/>
@@ -1469,10 +1501,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
@@ -1480,7 +1512,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B19" s="18" t="n">
         <f aca="false">B6/(10*(0.75+0.9+0.9+0.75)+2*8.5*0.75)</f>
@@ -1492,7 +1524,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="12" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1500,13 +1532,13 @@
         <v>3</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E22" s="3" t="s">
         <v>8</v>
@@ -1514,7 +1546,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B23" s="7" t="n">
         <v>254</v>
@@ -1534,7 +1566,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B24" s="7" t="n">
         <v>251.99</v>
@@ -1554,7 +1586,7 @@
     </row>
     <row r="25" s="14" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="14" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E25" s="15" t="n">
         <f aca="false">E23+E24</f>
@@ -1563,22 +1595,22 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
       <c r="D26" s="19" t="n">
-        <f aca="false">'Presupuesto equipo'!G11/B7</f>
-        <v>186.089189189189</v>
+        <f aca="false">'Presupuesto equipo'!G12/B7</f>
+        <v>199.690540540541</v>
       </c>
       <c r="E26" s="7" t="n">
-        <f aca="false">'Presupuesto equipo'!G11</f>
-        <v>6885.3</v>
+        <f aca="false">'Presupuesto equipo'!G12</f>
+        <v>7388.55</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="20" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B27" s="20"/>
       <c r="C27" s="20"/>
@@ -1618,12 +1650,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1631,7 +1663,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1639,7 +1671,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1647,7 +1679,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1655,7 +1687,7 @@
         <v>4</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1663,7 +1695,7 @@
         <v>5</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1671,7 +1703,7 @@
         <v>6</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1679,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1687,7 +1719,7 @@
         <v>8</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cimentación: placas de anclaje a 220 €/ud como material
12 placas a 220 € (2.640 €) en materiales; las 32 €/ud del equipo quedan
como colocación. Total por vivienda: 19.625,13 € sin IVA, también en
/cimentacion/.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UsshWDyzh9XkyW9ZdDTfjF
</commit_message>
<xml_diff>
--- a/costes/Nevola_cimentacion_presupuesto_equipo.xlsx
+++ b/costes/Nevola_cimentacion_presupuesto_equipo.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="99">
   <si>
     <t xml:space="preserve">Névola · Cimentación del piloto · Presupuesto del equipo</t>
   </si>
@@ -129,6 +129,12 @@
     <t xml:space="preserve">Los 3.000 kg, aparte de los 0,67 €/kg de elaboración y armado. Precio de Iván (20/10/2026)</t>
   </si>
   <si>
+    <t xml:space="preserve">Suministro de placas de anclaje</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Las 12 placas del presupuesto; la colocación va en mano de obra. Precio de Iván (20/10/2026)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Hormigón de limpieza bajo zapatas</t>
   </si>
   <si>
@@ -300,7 +306,7 @@
     <t xml:space="preserve">Canto de las zapatas: con 26 m³ sale ≈ 0,57 m. ¿Qué canto han previsto?</t>
   </si>
   <si>
-    <t xml:space="preserve">Placas: el croquis tiene 12 (3 por muro). En cada muro interior apoyan dos módulos y cada uno lleva su pilar, así que salen 2 placas por eje: 18 en total. ¿Las 32 € son por placa suministrada y colocada, con pernos?</t>
+    <t xml:space="preserve">Placas: el croquis tiene 12 (3 por muro). En cada muro interior apoyan dos módulos y cada uno lleva su pilar, así que salen 2 placas por eje: 18 en total. Las 32 € son la colocación; la placa se compra aparte a 220 €. ¿Incluye los pernos?</t>
   </si>
   <si>
     <t xml:space="preserve">Muretes transversales: 7,85 m en el croquis y 7,95 m en el cálculo. ¿Cuál es la buena?</t>
@@ -823,7 +829,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -1135,7 +1141,7 @@
         <v>2850</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4"/>
       <c r="B20" s="4" t="s">
         <v>35</v>
@@ -1144,22 +1150,21 @@
         <v>36</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E20" s="5" t="n">
-        <f aca="false">10*(0.75+0.9+0.9+0.75)+2*8.5*0.75</f>
-        <v>45.75</v>
+        <f aca="false">E10</f>
+        <v>12</v>
       </c>
       <c r="F20" s="6" t="n">
-        <f aca="false">0.1*F18</f>
-        <v>11.5</v>
+        <v>220</v>
       </c>
       <c r="G20" s="7" t="n">
         <f aca="false">IF(F20="","",E20*F20)</f>
-        <v>526.125</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>2640</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4"/>
       <c r="B21" s="4" t="s">
         <v>37</v>
@@ -1168,21 +1173,22 @@
         <v>38</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="E21" s="5" t="n">
-        <f aca="false">(10*(0.75+0.9+0.9+0.75)+2*8.5*0.75)*1.3</f>
-        <v>59.475</v>
+        <f aca="false">10*(0.75+0.9+0.9+0.75)+2*8.5*0.75</f>
+        <v>45.75</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>18</v>
+        <f aca="false">0.1*F18</f>
+        <v>11.5</v>
       </c>
       <c r="G21" s="7" t="n">
         <f aca="false">IF(F21="","",E21*F21)</f>
-        <v>1070.55</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>526.125</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4"/>
       <c r="B22" s="4" t="s">
         <v>39</v>
@@ -1191,21 +1197,21 @@
         <v>40</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="E22" s="5" t="n">
-        <f aca="false">7.85*9.5</f>
-        <v>74.575</v>
+        <f aca="false">(10*(0.75+0.9+0.9+0.75)+2*8.5*0.75)*1.3</f>
+        <v>59.475</v>
       </c>
       <c r="F22" s="6" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="G22" s="7" t="n">
         <f aca="false">IF(F22="","",E22*F22)</f>
-        <v>894.9</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1070.55</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4"/>
       <c r="B23" s="4" t="s">
         <v>41</v>
@@ -1214,13 +1220,18 @@
         <v>42</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="E23" s="5"/>
-      <c r="F23" s="6"/>
-      <c r="G23" s="7" t="str">
+        <v>25</v>
+      </c>
+      <c r="E23" s="5" t="n">
+        <f aca="false">7.85*9.5</f>
+        <v>74.575</v>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="G23" s="7" t="n">
         <f aca="false">IF(F23="","",E23*F23)</f>
-        <v/>
+        <v>894.9</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1241,22 +1252,40 @@
         <v/>
       </c>
     </row>
-    <row r="25" s="14" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="14" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4"/>
+      <c r="B25" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="G25" s="15" t="n">
-        <f aca="false">SUM(G18:G24)</f>
-        <v>9596.575</v>
-      </c>
-    </row>
-    <row r="26" s="8" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="9" t="s">
+      <c r="C25" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="G26" s="10" t="n">
-        <f aca="false">G12+G25</f>
-        <v>16985.125</v>
+      <c r="D25" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E25" s="5"/>
+      <c r="F25" s="6"/>
+      <c r="G25" s="7" t="str">
+        <f aca="false">IF(F25="","",E25*F25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" s="14" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="G26" s="15" t="n">
+        <f aca="false">SUM(G18:G25)</f>
+        <v>12236.575</v>
+      </c>
+    </row>
+    <row r="27" s="8" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B27" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="G27" s="10" t="n">
+        <f aca="false">G12+G26</f>
+        <v>19625.125</v>
       </c>
     </row>
   </sheetData>
@@ -1288,34 +1317,34 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B5" s="16" t="n">
         <f aca="false">'Presupuesto equipo'!E7</f>
@@ -1329,12 +1358,12 @@
         <v>2.42</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B6" s="16" t="n">
         <f aca="false">'Presupuesto equipo'!E8</f>
@@ -1348,12 +1377,12 @@
         <v>5.52</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B7" s="16" t="n">
         <f aca="false">B5+B6</f>
@@ -1371,7 +1400,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B8" s="17" t="n">
         <f aca="false">'Presupuesto equipo'!E9</f>
@@ -1385,12 +1414,12 @@
         <v>1333</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B9" s="16" t="n">
         <f aca="false">B8/B7</f>
@@ -1405,12 +1434,12 @@
         <v>23.7170067521066</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B10" s="17" t="n">
         <f aca="false">'Presupuesto equipo'!E10</f>
@@ -1424,12 +1453,12 @@
         <v>-6</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B11" s="16" t="n">
         <v>0.7</v>
@@ -1445,7 +1474,7 @@
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B12" s="16" t="n">
         <v>7.95</v>
@@ -1458,20 +1487,20 @@
         <v>1.05</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
@@ -1479,10 +1508,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C16" s="4"/>
       <c r="D16" s="4"/>
@@ -1490,10 +1519,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C17" s="4"/>
       <c r="D17" s="4"/>
@@ -1501,10 +1530,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
@@ -1512,7 +1541,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B19" s="18" t="n">
         <f aca="false">B6/(10*(0.75+0.9+0.9+0.75)+2*8.5*0.75)</f>
@@ -1524,7 +1553,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="12" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1532,13 +1561,13 @@
         <v>3</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E22" s="3" t="s">
         <v>8</v>
@@ -1546,7 +1575,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B23" s="7" t="n">
         <v>254</v>
@@ -1566,7 +1595,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B24" s="7" t="n">
         <v>251.99</v>
@@ -1586,7 +1615,7 @@
     </row>
     <row r="25" s="14" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="14" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E25" s="15" t="n">
         <f aca="false">E23+E24</f>
@@ -1595,7 +1624,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -1610,7 +1639,7 @@
     </row>
     <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="20" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B27" s="20"/>
       <c r="C27" s="20"/>
@@ -1650,12 +1679,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1663,7 +1692,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1671,7 +1700,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1679,7 +1708,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1687,7 +1716,7 @@
         <v>4</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1695,7 +1724,7 @@
         <v>5</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1703,7 +1732,7 @@
         <v>6</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1711,7 +1740,7 @@
         <v>7</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1719,7 +1748,7 @@
         <v>8</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cimentación: bombeo a 250 € por vivienda
Total por vivienda: 19.875,13 € sin IVA, también en /cimentacion/. Solo
queda fuera el replanteo topográfico.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UsshWDyzh9XkyW9ZdDTfjF
</commit_message>
<xml_diff>
--- a/costes/Nevola_cimentacion_presupuesto_equipo.xlsx
+++ b/costes/Nevola_cimentacion_presupuesto_equipo.xlsx
@@ -156,7 +156,7 @@
     <t xml:space="preserve">Bombeo de hormigón</t>
   </si>
   <si>
-    <t xml:space="preserve">Si hace falta en la parcela</t>
+    <t xml:space="preserve">Una partida por vivienda. Precio de Iván (20/10/2026)</t>
   </si>
   <si>
     <t xml:space="preserve">Replanteo topográfico</t>
@@ -1234,7 +1234,7 @@
         <v>894.9</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4"/>
       <c r="B24" s="4" t="s">
         <v>43</v>
@@ -1245,11 +1245,16 @@
       <c r="D24" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E24" s="5"/>
-      <c r="F24" s="6"/>
-      <c r="G24" s="7" t="str">
+      <c r="E24" s="5" t="n">
+        <f aca="false">1</f>
+        <v>1</v>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>250</v>
+      </c>
+      <c r="G24" s="7" t="n">
         <f aca="false">IF(F24="","",E24*F24)</f>
-        <v/>
+        <v>250</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1276,7 +1281,7 @@
       </c>
       <c r="G26" s="15" t="n">
         <f aca="false">SUM(G18:G25)</f>
-        <v>12236.575</v>
+        <v>12486.575</v>
       </c>
     </row>
     <row r="27" s="8" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1285,7 +1290,7 @@
       </c>
       <c r="G27" s="10" t="n">
         <f aca="false">G12+G26</f>
-        <v>19625.125</v>
+        <v>19875.125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cimentación: replanteo a 300 € por vivienda
Todas las partidas con precio: 20.175,13 € por vivienda sin IVA, también
en /cimentacion/ (desaparece la nota «No incluido»).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UsshWDyzh9XkyW9ZdDTfjF
</commit_message>
<xml_diff>
--- a/costes/Nevola_cimentacion_presupuesto_equipo.xlsx
+++ b/costes/Nevola_cimentacion_presupuesto_equipo.xlsx
@@ -162,7 +162,7 @@
     <t xml:space="preserve">Replanteo topográfico</t>
   </si>
   <si>
-    <t xml:space="preserve">Ejes de muros y placas</t>
+    <t xml:space="preserve">Ejes de muros y placas, por vivienda. Precio de Iván (20/10/2026)</t>
   </si>
   <si>
     <t xml:space="preserve">Subtotal de lo pendiente (solo lo que tenga precio)</t>
@@ -1257,7 +1257,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4"/>
       <c r="B25" s="4" t="s">
         <v>45</v>
@@ -1268,11 +1268,16 @@
       <c r="D25" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E25" s="5"/>
-      <c r="F25" s="6"/>
-      <c r="G25" s="7" t="str">
+      <c r="E25" s="5" t="n">
+        <f aca="false">1</f>
+        <v>1</v>
+      </c>
+      <c r="F25" s="6" t="n">
+        <v>300</v>
+      </c>
+      <c r="G25" s="7" t="n">
         <f aca="false">IF(F25="","",E25*F25)</f>
-        <v/>
+        <v>300</v>
       </c>
     </row>
     <row r="26" s="14" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1281,7 +1286,7 @@
       </c>
       <c r="G26" s="15" t="n">
         <f aca="false">SUM(G18:G25)</f>
-        <v>12486.575</v>
+        <v>12786.575</v>
       </c>
     </row>
     <row r="27" s="8" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1290,7 +1295,7 @@
       </c>
       <c r="G27" s="10" t="n">
         <f aca="false">G12+G26</f>
-        <v>19875.125</v>
+        <v>20175.125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>